<commit_message>
chore: regenerate demo Excel files with sub-levers sheet
</commit_message>
<xml_diff>
--- a/demo/leviers_demo.xlsx
+++ b/demo/leviers_demo.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Leviers" sheetId="1" r:id="rId1"/>
+    <sheet name="Sous-leviers" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -1147,4 +1148,176 @@
     <ignoredError numberStoredAsText="1" sqref="A1:AC8"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Levier Code</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Nom sous-levier</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Poste de dépense</v>
+      </c>
+      <c r="D1" t="str">
+        <v>BU</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Compte P&amp;L</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Impact brut (€M)</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Impact net (€M)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>AC-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Rationalisation fournisseurs packaging – Europe</v>
+      </c>
+      <c r="C2" t="str">
+        <v>COGS Packaging</v>
+      </c>
+      <c r="D2" t="str">
+        <v>BU Industrie</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Cost of Goods Sold</v>
+      </c>
+      <c r="F2">
+        <v>2.5</v>
+      </c>
+      <c r="G2">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>AC-001</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Rationalisation fournisseurs packaging – Asie</v>
+      </c>
+      <c r="C3" t="str">
+        <v>COGS Packaging APAC</v>
+      </c>
+      <c r="D3" t="str">
+        <v>BU Industrie</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Cost of Goods Sold</v>
+      </c>
+      <c r="F3">
+        <v>1.7</v>
+      </c>
+      <c r="G3">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>AC-002</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Maintenance prédictive lignes B1-B4</v>
+      </c>
+      <c r="C4" t="str">
+        <v>COGS Maintenance</v>
+      </c>
+      <c r="D4" t="str">
+        <v>BU Industrie</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Cost of Goods Sold</v>
+      </c>
+      <c r="F4">
+        <v>2.8</v>
+      </c>
+      <c r="G4">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>AC-003</v>
+      </c>
+      <c r="B5" t="str">
+        <v>RPA processus comptables</v>
+      </c>
+      <c r="C5" t="str">
+        <v>G&amp;A Finance</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Corporate</v>
+      </c>
+      <c r="E5" t="str">
+        <v>General &amp; Admin</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>AC-003</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Automatisation déclarations TVA</v>
+      </c>
+      <c r="C6" t="str">
+        <v>G&amp;A Tax</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Corporate</v>
+      </c>
+      <c r="E6" t="str">
+        <v>General &amp; Admin</v>
+      </c>
+      <c r="F6">
+        <v>0.5</v>
+      </c>
+      <c r="G6">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>AC-006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Transfert activités Mannheim → Rotterdam</v>
+      </c>
+      <c r="C7" t="str">
+        <v>COGS Logistique EMEA</v>
+      </c>
+      <c r="D7" t="str">
+        <v>BU Industrie</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Cost of Goods Sold</v>
+      </c>
+      <c r="F7">
+        <v>2.1</v>
+      </c>
+      <c r="G7">
+        <v>1.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: scope admin history to company, require company on Excel import, fix sub-lever demo headers
- admin/history: le journal d'audit affichait toutes les entreprises pour un
  admin_entreprise (aucun filtrage sur subscribeAuditLog). Ajout de
  filterAuditByCompany qui ne garde que les entrées liées aux leviers de la
  société courante.
- ExcelUploadButton: un import sans companyId (super-admin) attachait les
  leviers à aucune entreprise, les rendant visibles partout. Le sélecteur
  "Entreprise de destination" est désormais obligatoire dans ce cas.
- demo/leviers_demo.xlsx: la feuille "Sous-leviers" utilisait "Levier Code"/
  "BU" au lieu de "Code levier"/"Business Unit" et il manquait la moitié des
  colonnes lues par parseSubLeverExcelRow — chaque ligne était donc rejetée
  silencieusement à l'import (bouton "Confirmer" désactivé, aucun changement
  visible). Régénéré via generate-demo-excel.js avec les bons en-têtes.
</commit_message>
<xml_diff>
--- a/demo/leviers_demo.xlsx
+++ b/demo/leviers_demo.xlsx
@@ -1152,29 +1152,86 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:S7"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="17.83203125" customWidth="1"/>
+    <col min="9" max="9" width="19.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
+    <col min="13" max="13" width="21.83203125" customWidth="1"/>
+    <col min="14" max="14" width="16.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="14.83203125" customWidth="1"/>
+    <col min="18" max="18" width="14.83203125" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Levier Code</v>
+        <v>Code levier</v>
       </c>
       <c r="B1" t="str">
         <v>Nom sous-levier</v>
       </c>
       <c r="C1" t="str">
+        <v>Owner</v>
+      </c>
+      <c r="D1" t="str">
         <v>Poste de dépense</v>
       </c>
-      <c r="D1" t="str">
-        <v>BU</v>
-      </c>
       <c r="E1" t="str">
+        <v>Business Unit</v>
+      </c>
+      <c r="F1" t="str">
         <v>Compte P&amp;L</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Impact brut (€M)</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Impact net (€M)</v>
+      </c>
+      <c r="I1" t="str">
+        <v>OPEX one-off (€M)</v>
+      </c>
+      <c r="J1" t="str">
+        <v>OPEX récurrent (€M/an)</v>
+      </c>
+      <c r="K1" t="str">
+        <v>CAPEX (€M)</v>
+      </c>
+      <c r="L1" t="str">
+        <v>ETP</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Population impactée</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Date de départ</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Date de fin</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Statut</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Priorité</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Risque</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Dépendances</v>
       </c>
     </row>
     <row r="2">
@@ -1185,19 +1242,55 @@
         <v>Rationalisation fournisseurs packaging – Europe</v>
       </c>
       <c r="C2" t="str">
+        <v>Isabelle Roy</v>
+      </c>
+      <c r="D2" t="str">
         <v>COGS Packaging</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>BU Industrie</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>Cost of Goods Sold</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>2.5</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>2.2</v>
+      </c>
+      <c r="I2">
+        <v>0.2</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0.05</v>
+      </c>
+      <c r="L2">
+        <v>-2</v>
+      </c>
+      <c r="M2">
+        <v>80</v>
+      </c>
+      <c r="N2" t="str">
+        <v>2026-02-01</v>
+      </c>
+      <c r="O2" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="P2" t="str">
+        <v>L3 · Validé</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>high</v>
+      </c>
+      <c r="R2" t="str">
+        <v>medium</v>
+      </c>
+      <c r="S2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -1208,19 +1301,55 @@
         <v>Rationalisation fournisseurs packaging – Asie</v>
       </c>
       <c r="C3" t="str">
+        <v>Isabelle Roy</v>
+      </c>
+      <c r="D3" t="str">
         <v>COGS Packaging APAC</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>BU Industrie</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>Cost of Goods Sold</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>1.7</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>1.6</v>
+      </c>
+      <c r="I3">
+        <v>0.1</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0.05</v>
+      </c>
+      <c r="L3">
+        <v>-1</v>
+      </c>
+      <c r="M3">
+        <v>40</v>
+      </c>
+      <c r="N3" t="str">
+        <v>2026-03-01</v>
+      </c>
+      <c r="O3" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="P3" t="str">
+        <v>L2 · Qualifié</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>medium</v>
+      </c>
+      <c r="R3" t="str">
+        <v>medium</v>
+      </c>
+      <c r="S3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -1231,19 +1360,55 @@
         <v>Maintenance prédictive lignes B1-B4</v>
       </c>
       <c r="C4" t="str">
+        <v>Thomas Petit</v>
+      </c>
+      <c r="D4" t="str">
         <v>COGS Maintenance</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>BU Industrie</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>Cost of Goods Sold</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>2.8</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>2.5</v>
+      </c>
+      <c r="I4">
+        <v>0.2</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0.8</v>
+      </c>
+      <c r="L4">
+        <v>-5</v>
+      </c>
+      <c r="M4">
+        <v>340</v>
+      </c>
+      <c r="N4" t="str">
+        <v>2026-03-15</v>
+      </c>
+      <c r="O4" t="str">
+        <v>2026-12-31</v>
+      </c>
+      <c r="P4" t="str">
+        <v>L4 · Planifié</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>high</v>
+      </c>
+      <c r="R4" t="str">
+        <v>high</v>
+      </c>
+      <c r="S4" t="str">
+        <v>AC-001:SS</v>
       </c>
     </row>
     <row r="5">
@@ -1254,19 +1419,55 @@
         <v>RPA processus comptables</v>
       </c>
       <c r="C5" t="str">
+        <v>Claire Bernard</v>
+      </c>
+      <c r="D5" t="str">
         <v>G&amp;A Finance</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>Corporate</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>General &amp; Admin</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>1</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>0.8</v>
+      </c>
+      <c r="I5">
+        <v>0.3</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0.3</v>
+      </c>
+      <c r="L5">
+        <v>-2</v>
+      </c>
+      <c r="M5">
+        <v>25</v>
+      </c>
+      <c r="N5" t="str">
+        <v>2026-01-15</v>
+      </c>
+      <c r="O5" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="P5" t="str">
+        <v>L2 · Qualifié</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>medium</v>
+      </c>
+      <c r="R5" t="str">
+        <v>low</v>
+      </c>
+      <c r="S5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -1277,19 +1478,55 @@
         <v>Automatisation déclarations TVA</v>
       </c>
       <c r="C6" t="str">
+        <v>Claire Bernard</v>
+      </c>
+      <c r="D6" t="str">
         <v>G&amp;A Tax</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>Corporate</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>General &amp; Admin</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>0.5</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>0.4</v>
+      </c>
+      <c r="I6">
+        <v>0.1</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0.2</v>
+      </c>
+      <c r="L6">
+        <v>-2</v>
+      </c>
+      <c r="M6">
+        <v>20</v>
+      </c>
+      <c r="N6" t="str">
+        <v>2026-02-01</v>
+      </c>
+      <c r="O6" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="P6" t="str">
+        <v>L1 · Idée</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>medium</v>
+      </c>
+      <c r="R6" t="str">
+        <v>low</v>
+      </c>
+      <c r="S6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -1300,24 +1537,60 @@
         <v>Transfert activités Mannheim → Rotterdam</v>
       </c>
       <c r="C7" t="str">
+        <v>Marc Dubois</v>
+      </c>
+      <c r="D7" t="str">
         <v>COGS Logistique EMEA</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>BU Industrie</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <v>Cost of Goods Sold</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>2.1</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>1.8</v>
+      </c>
+      <c r="I7">
+        <v>0.5</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>1.2</v>
+      </c>
+      <c r="L7">
+        <v>-6</v>
+      </c>
+      <c r="M7">
+        <v>280</v>
+      </c>
+      <c r="N7" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="O7" t="str">
+        <v>2026-12-31</v>
+      </c>
+      <c r="P7" t="str">
+        <v>L3 · Validé</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>high</v>
+      </c>
+      <c r="R7" t="str">
+        <v>critical</v>
+      </c>
+      <c r="S7" t="str">
+        <v>AC-002:FS</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: scope admin history to company, require company on Excel import, fix sub-lever demo headers (#4)
- admin/history: le journal d'audit affichait toutes les entreprises pour un
  admin_entreprise (aucun filtrage sur subscribeAuditLog). Ajout de
  filterAuditByCompany qui ne garde que les entrées liées aux leviers de la
  société courante.
- ExcelUploadButton: un import sans companyId (super-admin) attachait les
  leviers à aucune entreprise, les rendant visibles partout. Le sélecteur
  "Entreprise de destination" est désormais obligatoire dans ce cas.
- demo/leviers_demo.xlsx: la feuille "Sous-leviers" utilisait "Levier Code"/
  "BU" au lieu de "Code levier"/"Business Unit" et il manquait la moitié des
  colonnes lues par parseSubLeverExcelRow — chaque ligne était donc rejetée
  silencieusement à l'import (bouton "Confirmer" désactivé, aucun changement
  visible). Régénéré via generate-demo-excel.js avec les bons en-têtes.
</commit_message>
<xml_diff>
--- a/demo/leviers_demo.xlsx
+++ b/demo/leviers_demo.xlsx
@@ -1152,29 +1152,86 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:S7"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="17.83203125" customWidth="1"/>
+    <col min="9" max="9" width="19.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
+    <col min="13" max="13" width="21.83203125" customWidth="1"/>
+    <col min="14" max="14" width="16.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="14.83203125" customWidth="1"/>
+    <col min="18" max="18" width="14.83203125" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Levier Code</v>
+        <v>Code levier</v>
       </c>
       <c r="B1" t="str">
         <v>Nom sous-levier</v>
       </c>
       <c r="C1" t="str">
+        <v>Owner</v>
+      </c>
+      <c r="D1" t="str">
         <v>Poste de dépense</v>
       </c>
-      <c r="D1" t="str">
-        <v>BU</v>
-      </c>
       <c r="E1" t="str">
+        <v>Business Unit</v>
+      </c>
+      <c r="F1" t="str">
         <v>Compte P&amp;L</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Impact brut (€M)</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Impact net (€M)</v>
+      </c>
+      <c r="I1" t="str">
+        <v>OPEX one-off (€M)</v>
+      </c>
+      <c r="J1" t="str">
+        <v>OPEX récurrent (€M/an)</v>
+      </c>
+      <c r="K1" t="str">
+        <v>CAPEX (€M)</v>
+      </c>
+      <c r="L1" t="str">
+        <v>ETP</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Population impactée</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Date de départ</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Date de fin</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Statut</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Priorité</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Risque</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Dépendances</v>
       </c>
     </row>
     <row r="2">
@@ -1185,19 +1242,55 @@
         <v>Rationalisation fournisseurs packaging – Europe</v>
       </c>
       <c r="C2" t="str">
+        <v>Isabelle Roy</v>
+      </c>
+      <c r="D2" t="str">
         <v>COGS Packaging</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>BU Industrie</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>Cost of Goods Sold</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>2.5</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>2.2</v>
+      </c>
+      <c r="I2">
+        <v>0.2</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0.05</v>
+      </c>
+      <c r="L2">
+        <v>-2</v>
+      </c>
+      <c r="M2">
+        <v>80</v>
+      </c>
+      <c r="N2" t="str">
+        <v>2026-02-01</v>
+      </c>
+      <c r="O2" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="P2" t="str">
+        <v>L3 · Validé</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>high</v>
+      </c>
+      <c r="R2" t="str">
+        <v>medium</v>
+      </c>
+      <c r="S2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -1208,19 +1301,55 @@
         <v>Rationalisation fournisseurs packaging – Asie</v>
       </c>
       <c r="C3" t="str">
+        <v>Isabelle Roy</v>
+      </c>
+      <c r="D3" t="str">
         <v>COGS Packaging APAC</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>BU Industrie</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>Cost of Goods Sold</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>1.7</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>1.6</v>
+      </c>
+      <c r="I3">
+        <v>0.1</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0.05</v>
+      </c>
+      <c r="L3">
+        <v>-1</v>
+      </c>
+      <c r="M3">
+        <v>40</v>
+      </c>
+      <c r="N3" t="str">
+        <v>2026-03-01</v>
+      </c>
+      <c r="O3" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="P3" t="str">
+        <v>L2 · Qualifié</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>medium</v>
+      </c>
+      <c r="R3" t="str">
+        <v>medium</v>
+      </c>
+      <c r="S3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -1231,19 +1360,55 @@
         <v>Maintenance prédictive lignes B1-B4</v>
       </c>
       <c r="C4" t="str">
+        <v>Thomas Petit</v>
+      </c>
+      <c r="D4" t="str">
         <v>COGS Maintenance</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>BU Industrie</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>Cost of Goods Sold</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>2.8</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>2.5</v>
+      </c>
+      <c r="I4">
+        <v>0.2</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0.8</v>
+      </c>
+      <c r="L4">
+        <v>-5</v>
+      </c>
+      <c r="M4">
+        <v>340</v>
+      </c>
+      <c r="N4" t="str">
+        <v>2026-03-15</v>
+      </c>
+      <c r="O4" t="str">
+        <v>2026-12-31</v>
+      </c>
+      <c r="P4" t="str">
+        <v>L4 · Planifié</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>high</v>
+      </c>
+      <c r="R4" t="str">
+        <v>high</v>
+      </c>
+      <c r="S4" t="str">
+        <v>AC-001:SS</v>
       </c>
     </row>
     <row r="5">
@@ -1254,19 +1419,55 @@
         <v>RPA processus comptables</v>
       </c>
       <c r="C5" t="str">
+        <v>Claire Bernard</v>
+      </c>
+      <c r="D5" t="str">
         <v>G&amp;A Finance</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>Corporate</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>General &amp; Admin</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>1</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>0.8</v>
+      </c>
+      <c r="I5">
+        <v>0.3</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0.3</v>
+      </c>
+      <c r="L5">
+        <v>-2</v>
+      </c>
+      <c r="M5">
+        <v>25</v>
+      </c>
+      <c r="N5" t="str">
+        <v>2026-01-15</v>
+      </c>
+      <c r="O5" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="P5" t="str">
+        <v>L2 · Qualifié</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>medium</v>
+      </c>
+      <c r="R5" t="str">
+        <v>low</v>
+      </c>
+      <c r="S5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -1277,19 +1478,55 @@
         <v>Automatisation déclarations TVA</v>
       </c>
       <c r="C6" t="str">
+        <v>Claire Bernard</v>
+      </c>
+      <c r="D6" t="str">
         <v>G&amp;A Tax</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>Corporate</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>General &amp; Admin</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>0.5</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>0.4</v>
+      </c>
+      <c r="I6">
+        <v>0.1</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0.2</v>
+      </c>
+      <c r="L6">
+        <v>-2</v>
+      </c>
+      <c r="M6">
+        <v>20</v>
+      </c>
+      <c r="N6" t="str">
+        <v>2026-02-01</v>
+      </c>
+      <c r="O6" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="P6" t="str">
+        <v>L1 · Idée</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>medium</v>
+      </c>
+      <c r="R6" t="str">
+        <v>low</v>
+      </c>
+      <c r="S6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -1300,24 +1537,60 @@
         <v>Transfert activités Mannheim → Rotterdam</v>
       </c>
       <c r="C7" t="str">
+        <v>Marc Dubois</v>
+      </c>
+      <c r="D7" t="str">
         <v>COGS Logistique EMEA</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>BU Industrie</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <v>Cost of Goods Sold</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>2.1</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>1.8</v>
+      </c>
+      <c r="I7">
+        <v>0.5</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>1.2</v>
+      </c>
+      <c r="L7">
+        <v>-6</v>
+      </c>
+      <c r="M7">
+        <v>280</v>
+      </c>
+      <c r="N7" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="O7" t="str">
+        <v>2026-12-31</v>
+      </c>
+      <c r="P7" t="str">
+        <v>L3 · Validé</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>high</v>
+      </c>
+      <c r="R7" t="str">
+        <v>critical</v>
+      </c>
+      <c r="S7" t="str">
+        <v>AC-002:FS</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: align lever Excel import/export with the actually displayed lifecycle labels
DEFAULT_LIFECYCLE_STAGES (short labels: "Identifié", "Validé"...) is
always what's shown on screen (Kanban, status dropdowns, stepper),
but the Excel import/export used a separate, unsynchronized static
dictionary (STATUS_LABEL, long labels: "Levier identifié", "Business
case validé"...). Re-importing the demo file — or exporting a
company's levers and re-importing that file — failed with "Statut
inconnu" errors.

Import now validates the "Statut" column against the union of
short/long/company-specific labels; export now writes the label
actually shown on screen. Demo file regenerated via the existing
scripts/generate-demo-excel.js so it stays in sync going forward.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/leviers_demo.xlsx
+++ b/demo/leviers_demo.xlsx
@@ -540,7 +540,7 @@
         <v>2026-06-28</v>
       </c>
       <c r="R2" t="str">
-        <v>Levier identifié</v>
+        <v>Identifié</v>
       </c>
       <c r="S2">
         <v>0</v>
@@ -626,7 +626,7 @@
         <v>2026-08-28</v>
       </c>
       <c r="R3" t="str">
-        <v>Business case validé</v>
+        <v>Validé</v>
       </c>
       <c r="S3">
         <v>0</v>
@@ -712,7 +712,7 @@
         <v>2026-10-28</v>
       </c>
       <c r="R4" t="str">
-        <v>Implémentation planifiée</v>
+        <v>Planifié</v>
       </c>
       <c r="S4">
         <v>15</v>
@@ -798,7 +798,7 @@
         <v>2026-12-28</v>
       </c>
       <c r="R5" t="str">
-        <v>En cours d'exécution</v>
+        <v>Exécuté</v>
       </c>
       <c r="S5">
         <v>55</v>
@@ -884,7 +884,7 @@
         <v>2027-02-28</v>
       </c>
       <c r="R6" t="str">
-        <v>Valeur réalisée</v>
+        <v>Réalisé</v>
       </c>
       <c r="S6">
         <v>100</v>
@@ -970,7 +970,7 @@
         <v>2027-04-28</v>
       </c>
       <c r="R7" t="str">
-        <v>Levier identifié</v>
+        <v>Identifié</v>
       </c>
       <c r="S7">
         <v>0</v>
@@ -1056,7 +1056,7 @@
         <v>2027-06-28</v>
       </c>
       <c r="R8" t="str">
-        <v>Business case validé</v>
+        <v>Validé</v>
       </c>
       <c r="S8">
         <v>0</v>
@@ -1142,7 +1142,7 @@
         <v>2027-08-28</v>
       </c>
       <c r="R9" t="str">
-        <v>Implémentation planifiée</v>
+        <v>Planifié</v>
       </c>
       <c r="S9">
         <v>10</v>
@@ -1228,7 +1228,7 @@
         <v>2027-02-28</v>
       </c>
       <c r="R10" t="str">
-        <v>En cours d'exécution</v>
+        <v>Exécuté</v>
       </c>
       <c r="S10">
         <v>45</v>
@@ -1314,7 +1314,7 @@
         <v>2027-04-28</v>
       </c>
       <c r="R11" t="str">
-        <v>Valeur réalisée</v>
+        <v>Réalisé</v>
       </c>
       <c r="S11">
         <v>100</v>
@@ -1400,7 +1400,7 @@
         <v>2026-08-28</v>
       </c>
       <c r="R12" t="str">
-        <v>Levier identifié</v>
+        <v>Identifié</v>
       </c>
       <c r="S12">
         <v>0</v>
@@ -1486,7 +1486,7 @@
         <v>2026-10-28</v>
       </c>
       <c r="R13" t="str">
-        <v>Business case validé</v>
+        <v>Validé</v>
       </c>
       <c r="S13">
         <v>0</v>
@@ -1572,7 +1572,7 @@
         <v>2026-12-28</v>
       </c>
       <c r="R14" t="str">
-        <v>Implémentation planifiée</v>
+        <v>Planifié</v>
       </c>
       <c r="S14">
         <v>5</v>
@@ -1658,7 +1658,7 @@
         <v>2027-02-28</v>
       </c>
       <c r="R15" t="str">
-        <v>En cours d'exécution</v>
+        <v>Exécuté</v>
       </c>
       <c r="S15">
         <v>35</v>
@@ -1744,7 +1744,7 @@
         <v>2027-04-28</v>
       </c>
       <c r="R16" t="str">
-        <v>Valeur réalisée</v>
+        <v>Réalisé</v>
       </c>
       <c r="S16">
         <v>100</v>
@@ -1830,7 +1830,7 @@
         <v>2027-06-28</v>
       </c>
       <c r="R17" t="str">
-        <v>Levier identifié</v>
+        <v>Identifié</v>
       </c>
       <c r="S17">
         <v>0</v>
@@ -1916,7 +1916,7 @@
         <v>2026-12-28</v>
       </c>
       <c r="R18" t="str">
-        <v>Business case validé</v>
+        <v>Validé</v>
       </c>
       <c r="S18">
         <v>0</v>
@@ -2002,7 +2002,7 @@
         <v>2027-02-28</v>
       </c>
       <c r="R19" t="str">
-        <v>Implémentation planifiée</v>
+        <v>Planifié</v>
       </c>
       <c r="S19">
         <v>15</v>
@@ -2088,7 +2088,7 @@
         <v>2027-04-28</v>
       </c>
       <c r="R20" t="str">
-        <v>En cours d'exécution</v>
+        <v>Exécuté</v>
       </c>
       <c r="S20">
         <v>25</v>
@@ -2174,7 +2174,7 @@
         <v>2027-06-28</v>
       </c>
       <c r="R21" t="str">
-        <v>Valeur réalisée</v>
+        <v>Réalisé</v>
       </c>
       <c r="S21">
         <v>100</v>
@@ -2260,7 +2260,7 @@
         <v>2026-10-28</v>
       </c>
       <c r="R22" t="str">
-        <v>Levier identifié</v>
+        <v>Identifié</v>
       </c>
       <c r="S22">
         <v>0</v>
@@ -2346,7 +2346,7 @@
         <v>2026-12-28</v>
       </c>
       <c r="R23" t="str">
-        <v>Business case validé</v>
+        <v>Validé</v>
       </c>
       <c r="S23">
         <v>0</v>
@@ -2432,7 +2432,7 @@
         <v>2027-02-28</v>
       </c>
       <c r="R24" t="str">
-        <v>Implémentation planifiée</v>
+        <v>Planifié</v>
       </c>
       <c r="S24">
         <v>10</v>
@@ -2518,7 +2518,7 @@
         <v>2027-04-28</v>
       </c>
       <c r="R25" t="str">
-        <v>En cours d'exécution</v>
+        <v>Exécuté</v>
       </c>
       <c r="S25">
         <v>75</v>
@@ -2604,7 +2604,7 @@
         <v>2026-10-28</v>
       </c>
       <c r="R26" t="str">
-        <v>Valeur réalisée</v>
+        <v>Réalisé</v>
       </c>
       <c r="S26">
         <v>100</v>
@@ -2690,7 +2690,7 @@
         <v>2026-12-28</v>
       </c>
       <c r="R27" t="str">
-        <v>Levier identifié</v>
+        <v>Identifié</v>
       </c>
       <c r="S27">
         <v>0</v>
@@ -2776,7 +2776,7 @@
         <v>2027-02-28</v>
       </c>
       <c r="R28" t="str">
-        <v>Business case validé</v>
+        <v>Validé</v>
       </c>
       <c r="S28">
         <v>0</v>
@@ -2862,7 +2862,7 @@
         <v>2027-04-28</v>
       </c>
       <c r="R29" t="str">
-        <v>Implémentation planifiée</v>
+        <v>Planifié</v>
       </c>
       <c r="S29">
         <v>5</v>
@@ -2948,7 +2948,7 @@
         <v>2027-06-28</v>
       </c>
       <c r="R30" t="str">
-        <v>En cours d'exécution</v>
+        <v>Exécuté</v>
       </c>
       <c r="S30">
         <v>65</v>
@@ -3034,7 +3034,7 @@
         <v>2027-08-28</v>
       </c>
       <c r="R31" t="str">
-        <v>Valeur réalisée</v>
+        <v>Réalisé</v>
       </c>
       <c r="S31">
         <v>100</v>

</xml_diff>